<commit_message>
add SING-2B-002, SING-3B-001, COR-2B-001, COR-3B-002, XTHR-3B-002
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database.xlsx
+++ b/database.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,6 +36,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="11">
@@ -134,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -196,6 +200,9 @@
     <xf numFmtId="0" fontId="2" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -295,6 +302,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -320,6 +330,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -345,6 +358,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -370,6 +386,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -395,6 +414,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -420,6 +442,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -716,7 +741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -905,129 +930,321 @@
       </c>
     </row>
     <row r="5" ht="130" customHeight="1">
-      <c r="A5" s="21" t="n"/>
-      <c r="B5" s="22" t="inlineStr">
-        <is>
-          <t>COR-3B-001</t>
-        </is>
-      </c>
-      <c r="C5" s="22" t="n">
-        <v>3</v>
-      </c>
-      <c r="D5" s="22" t="n">
-        <v>2</v>
-      </c>
-      <c r="E5" s="22" t="inlineStr">
-        <is>
-          <t>Corner</t>
-        </is>
-      </c>
-      <c r="F5" s="22" t="n">
-        <v>10</v>
-      </c>
-      <c r="G5" s="22" t="n"/>
-      <c r="H5" s="21" t="n">
-        <v>12.7</v>
-      </c>
-      <c r="I5" s="21" t="inlineStr">
-        <is>
-          <t>2399 Redfern Comp APT 401</t>
-        </is>
-      </c>
-      <c r="J5" t="n">
-        <v>100.85</v>
-      </c>
-      <c r="K5" t="inlineStr">
+      <c r="A5" s="27" t="n"/>
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>SING-2B-002</t>
+        </is>
+      </c>
+      <c r="C5" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" s="24" t="inlineStr">
+        <is>
+          <t>Single aspect</t>
+        </is>
+      </c>
+      <c r="F5" s="24" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="G5" s="24" t="n"/>
+      <c r="H5" s="27" t="n">
+        <v>9.449999999999999</v>
+      </c>
+      <c r="I5" s="27" t="inlineStr">
+        <is>
+          <t>2101 Midtown, Macquarie Park APT 701</t>
+        </is>
+      </c>
+      <c r="J5" s="27" t="n">
+        <v>82.5</v>
+      </c>
+      <c r="K5" s="27" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="6" ht="130" customHeight="1">
-      <c r="A6" s="13" t="n"/>
-      <c r="B6" s="14" t="inlineStr">
-        <is>
-          <t>XTHR-2B-001</t>
-        </is>
-      </c>
-      <c r="C6" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="D6" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>Cross-through</t>
-        </is>
-      </c>
-      <c r="F6" s="14" t="n">
-        <v>6.6</v>
-      </c>
-      <c r="G6" s="14" t="n"/>
-      <c r="H6" s="13" t="n">
-        <v>14.45</v>
-      </c>
-      <c r="I6" s="15" t="inlineStr">
-        <is>
-          <t>1405 Rochford, Erskineville</t>
-        </is>
-      </c>
-      <c r="J6" t="n">
-        <v>76.11</v>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="A6" s="27" t="n"/>
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>SING-3B-001</t>
+        </is>
+      </c>
+      <c r="C6" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="24" t="inlineStr">
+        <is>
+          <t>Single aspect</t>
+        </is>
+      </c>
+      <c r="F6" s="24" t="n">
+        <v>13.65</v>
+      </c>
+      <c r="G6" s="24" t="n"/>
+      <c r="H6" s="27" t="n">
+        <v>9.449999999999999</v>
+      </c>
+      <c r="I6" s="27" t="inlineStr">
+        <is>
+          <t>2101 Midtown, Macquarie Park APT 801</t>
+        </is>
+      </c>
+      <c r="J6" s="27" t="n">
+        <v>98.52</v>
+      </c>
+      <c r="K6" s="27" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="7" ht="130" customHeight="1">
-      <c r="A7" s="25" t="n"/>
-      <c r="B7" s="26" t="inlineStr">
+      <c r="A7" s="28" t="n"/>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>COR-2B-001</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="22" t="inlineStr">
+        <is>
+          <t>Corner</t>
+        </is>
+      </c>
+      <c r="F7" s="22" t="n">
+        <v>8.35</v>
+      </c>
+      <c r="G7" s="22" t="n"/>
+      <c r="H7" s="28" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="I7" s="28" t="inlineStr">
+        <is>
+          <t>TYPICAL</t>
+        </is>
+      </c>
+      <c r="J7" s="28" t="n">
+        <v>77.19</v>
+      </c>
+      <c r="K7" s="28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="130" customHeight="1">
+      <c r="A8" s="21" t="n"/>
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>COR-3B-001</t>
+        </is>
+      </c>
+      <c r="C8" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="D8" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" s="22" t="inlineStr">
+        <is>
+          <t>Corner</t>
+        </is>
+      </c>
+      <c r="F8" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G8" s="22" t="n"/>
+      <c r="H8" s="21" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="I8" s="21" t="inlineStr">
+        <is>
+          <t>2399 Redfern Comp APT 401</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>100.85</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="130" customHeight="1">
+      <c r="A9" s="28" t="n"/>
+      <c r="B9" s="22" t="inlineStr">
+        <is>
+          <t>COR-3B-002</t>
+        </is>
+      </c>
+      <c r="C9" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" s="22" t="inlineStr">
+        <is>
+          <t>Corner</t>
+        </is>
+      </c>
+      <c r="F9" s="22" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="G9" s="22" t="n"/>
+      <c r="H9" s="28" t="n">
+        <v>15.05</v>
+      </c>
+      <c r="I9" s="28" t="inlineStr">
+        <is>
+          <t>2408 Kingsford APT 901</t>
+        </is>
+      </c>
+      <c r="J9" s="28" t="n">
+        <v>115.06</v>
+      </c>
+      <c r="K9" s="28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="130" customHeight="1">
+      <c r="A10" s="13" t="n"/>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>XTHR-2B-001</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>Cross-through</t>
+        </is>
+      </c>
+      <c r="F10" s="14" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="G10" s="14" t="n"/>
+      <c r="H10" s="13" t="n">
+        <v>14.45</v>
+      </c>
+      <c r="I10" s="15" t="inlineStr">
+        <is>
+          <t>1405 Rochford, Erskineville</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>76.11</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="130" customHeight="1">
+      <c r="A11" s="25" t="n"/>
+      <c r="B11" s="26" t="inlineStr">
         <is>
           <t>XTHR-2B-002</t>
         </is>
       </c>
-      <c r="C7" s="26" t="n">
-        <v>2</v>
-      </c>
-      <c r="D7" s="26" t="n">
-        <v>2</v>
-      </c>
-      <c r="E7" s="26" t="inlineStr">
+      <c r="C11" s="26" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" s="26" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" s="26" t="inlineStr">
         <is>
           <t>Cross-through</t>
         </is>
       </c>
-      <c r="F7" s="26" t="n">
+      <c r="F11" s="26" t="n">
         <v>6.85</v>
       </c>
-      <c r="G7" s="26" t="n">
+      <c r="G11" s="26" t="n">
         <v>4.3</v>
       </c>
-      <c r="H7" s="25" t="n">
+      <c r="H11" s="25" t="n">
         <v>17.35</v>
       </c>
-      <c r="I7" s="25" t="inlineStr">
+      <c r="I11" s="25" t="inlineStr">
         <is>
           <t>2101 Midtown, Macquarie Park APT 501</t>
         </is>
       </c>
-      <c r="J7" t="n">
+      <c r="J11" t="n">
         <v>83.5</v>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="130" customHeight="1"/>
-    <row r="9" ht="130" customHeight="1"/>
-    <row r="10" ht="130" customHeight="1"/>
-    <row r="11" ht="130" customHeight="1"/>
-    <row r="12" ht="130" customHeight="1"/>
+    <row r="12" ht="130" customHeight="1">
+      <c r="A12" s="29" t="n"/>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>XTHR-3B-002</t>
+        </is>
+      </c>
+      <c r="C12" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" s="26" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" s="26" t="inlineStr">
+        <is>
+          <t>Cross-through</t>
+        </is>
+      </c>
+      <c r="F12" s="26" t="n">
+        <v>10</v>
+      </c>
+      <c r="G12" s="26" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="H12" s="29" t="n">
+        <v>17.35</v>
+      </c>
+      <c r="I12" s="29" t="inlineStr">
+        <is>
+          <t>2101 Midtown, Macquarie Park APT 1201</t>
+        </is>
+      </c>
+      <c r="J12" s="29" t="n">
+        <v>98.31</v>
+      </c>
+      <c r="K12" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
     <row r="13" ht="130" customHeight="1"/>
     <row r="14" ht="130" customHeight="1"/>
     <row r="15" ht="130" customHeight="1"/>

</xml_diff>